<commit_message>
Move the counter prototype into the app, with a no-accounts demo mode
- The prototype screen is now the home page (components/counter), loading
  stock from /api/counter/inventory and vehicles from /api/counter/vehicle.
- Demo mode (no SUPABASE_URL, or DEMO_MODE=1): sample fitment plus the demo
  sheet run through the real cleaner; /sync previews the Sync issues tab.
- Live mode: Supabase inventory and shop_settings fees, fitment through the
  Wheel-Size cache, settled searches logged to counter_searches.
- Vehicle and fitment lookups moved out of their routes into lib/ so the
  routes and the counter share them.
- demo/demo-inventory.json is the single source for the demo sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01553HyVVidBZdxd6kDcsZdf
</commit_message>
<xml_diff>
--- a/demo/demo-inventory.xlsx
+++ b/demo/demo-inventory.xlsx
@@ -563,7 +563,6 @@
           <t>Rack B-04</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -613,7 +612,6 @@
           <t>Rack B-05</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -663,7 +661,6 @@
           <t>Rack B-06</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -771,7 +768,6 @@
           <t>Rack C-02</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -821,7 +817,6 @@
           <t>Rack C-03</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -925,7 +920,6 @@
           <t>Rack C-07</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -979,7 +973,6 @@
           <t>Used U-12</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1029,7 +1022,6 @@
           <t>Rack A-05</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1195,7 +1187,6 @@
           <t>Rack A-09</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1245,7 +1236,6 @@
           <t>Rack A-12</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1295,7 +1285,6 @@
           <t>Rack A-02</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1345,7 +1334,6 @@
           <t>Yard 1</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1395,7 +1383,6 @@
           <t>Yard 1</t>
         </is>
       </c>
-      <c r="L19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1445,7 +1432,6 @@
           <t>Yard 2</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1495,7 +1481,6 @@
           <t>Yard 3</t>
         </is>
       </c>
-      <c r="L21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Show staggered fitments as front + rear pairs
Wheel-Size's rear axle was dropped, so staggered cars (X3 M, Mustang...)
showed only front sizes. Each OE entry now carries its rear size, load,
speed, rim width and offset; a different rear is a different fitment.

The counter shows one card per staggered fitment (front and rear with
stock counts and both rims), lists front and rear tires in their own
groups, never offers the other axle's size as an alternate, and quotes a
pair per axle (front + rear, front pair or rear pair). Rear rims count as
OE for wheel matching. Special order shows per axle.

Demo: X3 M is staggered, with a staggered set in the demo stock.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01553HyVVidBZdxd6kDcsZdf
</commit_message>
<xml_diff>
--- a/demo/demo-inventory.xlsx
+++ b/demo/demo-inventory.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1645,6 +1645,114 @@
       <c r="L24" s="3" t="inlineStr">
         <is>
           <t>qty typed as a word: not synced</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>255/45R20</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Michelin</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Pilot Sport 4S</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Summer</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>105Y</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>1525</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" t="n">
+        <v>389</v>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Rack C-01</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>staggered front (X3 M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>265/45R20</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Michelin</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Pilot Sport 4S</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Summer</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr"/>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>108Y</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>1525</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" t="n">
+        <v>409</v>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Rack C-01</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>staggered rear (X3 M)</t>
         </is>
       </c>
     </row>

</xml_diff>